<commit_message>
update document desriptions manual reviews
</commit_message>
<xml_diff>
--- a/Document_descriptions_reviews.xlsx
+++ b/Document_descriptions_reviews.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Progetti_IA\Renco\kickoff\Script python\riconciliazione_mdr_1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE1270A-36D7-4212-A77A-5D439B42B4FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33E47C8A-5316-4753-8CBF-806128BE4F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>CONTROL AND SAFEGUARDING SYSTEMS ARCHITECTURE</t>
   </si>
@@ -180,9 +191,6 @@
     <t>PIPING COMPONENTS AND VALVES TECHNICAL SPECIFICATIONS</t>
   </si>
   <si>
-    <t>Technical specification for piping components and valves, defining functional requirements, materials, pressure-temperature ratings, end connections, testing, inspection and vendor documentation deliverables.</t>
-  </si>
-  <si>
     <t>PIPING TIE-INS LIST</t>
   </si>
   <si>
@@ -198,9 +206,6 @@
     <t>SUPPORT MATERIAL LIST</t>
   </si>
   <si>
-    <t>Support material list listing required materials, sizes, quantities and basic specifications for piping supports in PIPING SUPPORTS; prepared for procurement and require EMPLOYER approval.</t>
-  </si>
-  <si>
     <t>TECHNICAL DATA SHEETS FOR SPECIAL ITEM</t>
   </si>
   <si>
@@ -222,9 +227,6 @@
     <t>TECHNICAL SPECIFICATION FOR PURCHASE/HANDLING OF CONSUMABLES</t>
   </si>
   <si>
-    <t>Specification for purchase and handling of consumables, defining approved consumable types, storage, handling, traceability, inspection, and documentation requirements relevant to welding activities in the WELDING chapter.</t>
-  </si>
-  <si>
     <t>TYPICAL PIPING ASSEMBLY DRAWING</t>
   </si>
   <si>
@@ -271,6 +273,27 @@
   </si>
   <si>
     <t>Inspection checklist for HV switchgear, recording visual inspection, insulation resistance, mechanical operation, control circuit checks, interlocks, protection relay tests, and vendor factory documentation for acceptance.</t>
+  </si>
+  <si>
+    <t>ANALISI FEM DEI PONTI TERMICI (SOLO COMMESSE ITA, EDIFICI NUOVI)</t>
+  </si>
+  <si>
+    <t>Finite Element Method (FEM) modelling of building envelope junctions to evaluate thermal bridges in new buildings located in Italy. The analysis determines linear thermal transmittance (Ψ-values) in accordance with UNI EN ISO 10211 and the Italian “Decreto Requisiti Minimi”, and verifies internal surface temperatures to prevent mould and condensation.</t>
+  </si>
+  <si>
+    <t>HEATING AND COOLING PIPING AND EQUIPMENTS LAYOUTS</t>
+  </si>
+  <si>
+    <t>Layout drawings showing routing and pipe sizing of heating and cooling piping systems, equipment locations, valves, insulation specification, supports and maintenance clearances, including schedules for construction.</t>
+  </si>
+  <si>
+    <t>Technical specifications for piping components and valves, defining functional requirements, materials, pressure-temperature ratings, end connections, testing, inspection and vendor documentation deliverables.</t>
+  </si>
+  <si>
+    <t>Support material list listing required materials, sizes, quantities and basic specifications for piping supports in PIPING SUPPORTS; prepared for procurement and does NOT require EMPLOYER approval.</t>
+  </si>
+  <si>
+    <t>Specification for purchase and handling of consumables, defining approved consumable types, storage, handling, traceability, inspection, certification review, and documentation requirements relevant to welding activities in the WELDING chapter.</t>
   </si>
 </sst>
 </file>
@@ -591,10 +614,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="47.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="58.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="66.5546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
@@ -669,260 +693,276 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+    <row r="15" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+    <row r="19" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+    <row r="20" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B20" s="1" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="1" t="s">
+    </row>
+    <row r="30" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="B30" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="1" t="s">
+    </row>
+    <row r="31" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
+      <c r="B31" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+    <row r="33" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+    <row r="34" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="72" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="1" t="s">
+    </row>
+    <row r="43" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>